<commit_message>
DEC-019: Playwright pinned at 1.64.0 (ADR and Decision Log v0.8 H23)
</commit_message>
<xml_diff>
--- a/docs/decisions/Decision Log/Decision Log v0.8.xlsx
+++ b/docs/decisions/Decision Log/Decision Log v0.8.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huawei\Desktop\SEN381\Ticketing-System\docs\decisions\Decision Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B994036-69EA-4B15-A624-A6A4B485E87D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F7CD74-8BAF-42BC-AF5A-007286DD943D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13200" yWindow="0" windowWidth="13543" windowHeight="17829" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-86" yWindow="0" windowWidth="13543" windowHeight="17914" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Decision Log" sheetId="1" r:id="rId1"/>
@@ -404,10 +404,10 @@
     <t>DEC-003's deploy procedure has no client build step: a procedure gap for R. van der Merwe at staging time, closed by a new DEC-003 version. eslint.config.js needs a client/ block (browser globals, JSX) once #89 is updated from dev. CI does not build the client. NFR-1.1 browser coverage not claimed (Chromium only). The E2E specs are held until PR #88 merges, because they reuse its fixture harness</t>
   </si>
   <si>
-    <t>Pinned Playwright version when e2e/ lands; a recorded local E2E run (E2E-1 and E2E-2a pass, E2E-2b an expected failure with its 422 quoted); the client build step in DEC-003 before the staging run</t>
-  </si>
-  <si>
     <t>Decisions and deferments taken during M1, M2 and M3, the alternatives weighed, and what each one commits or blocks downstream</t>
+  </si>
+  <si>
+    <t>Playwright pinned at @playwright/test 1.64.0 (exact, e2e/package.json; Chromium build 1248). Still required: a recorded local E2E run (E2E-1 and E2E-2a pass, E2E-2b an expected failure with its 422 quoted); the client build step in DEC-003 before the staging run.</t>
   </si>
 </sst>
 </file>
@@ -1100,7 +1100,7 @@
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.4">
       <c r="B2" s="26" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C2" s="23"/>
       <c r="D2" s="23"/>
@@ -1796,7 +1796,7 @@
         <v>122</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I23" s="11" t="s">
         <v>18</v>

</xml_diff>